<commit_message>
fixed sponsors cards, updated first year guide, updates events and opportunities
</commit_message>
<xml_diff>
--- a/src/data/events_template.xlsx
+++ b/src/data/events_template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="240">
   <si>
     <t>Field</t>
   </si>
@@ -634,19 +634,28 @@
     <t>Coffee availble for purchase on a society tab</t>
   </si>
   <si>
-    <t>SUDATA Pub Crawl</t>
+    <t>SUDATA x SUMS x EconSoc Trivia &amp; Pub Crawl</t>
+  </si>
+  <si>
+    <t>BHB Seminar Room 3200</t>
+  </si>
+  <si>
+    <t>A social night out hopping between venues with SUDATA, SUMS and EconSoc members to unwind and meet new people</t>
+  </si>
+  <si>
+    <t>SUDATA, SUMS, Econsoc</t>
+  </si>
+  <si>
+    <t>Food provided at the Trivia</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLScqpPcQ59sVttaKaBFjwePnOLHKFWUo0syGt0UPCwH8KmnG5A/viewform?usp=dialog</t>
+  </si>
+  <si>
+    <t>Total Drama Island 2026 Camp</t>
   </si>
   <si>
     <t>TBD</t>
-  </si>
-  <si>
-    <t>A social night out hopping between venues with SUDATA members to unwind and meet new people</t>
-  </si>
-  <si>
-    <t>Drinks available for purchase</t>
-  </si>
-  <si>
-    <t>Total Drama Island 2026 Camp</t>
   </si>
   <si>
     <t>Great Aussie Bush Camp Lake Macquarie (Morisset)</t>
@@ -759,7 +768,7 @@
     <numFmt numFmtId="165" formatCode="hh:mm"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -788,6 +797,12 @@
       <sz val="11.0"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11.0"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
@@ -861,7 +876,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -895,46 +910,49 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -2885,11 +2903,11 @@
       <c r="B5" s="7">
         <v>46101.0</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4">
+        <v>0.7291666666666666</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>202</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>30</v>
@@ -2898,78 +2916,78 @@
         <v>203</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>32</v>
+        <v>204</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>35</v>
+        <v>205</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B6" s="7">
         <v>46108.0</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>30</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="I6" s="11" t="s">
-        <v>209</v>
+      <c r="I6" s="12" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="12">
+        <v>213</v>
+      </c>
+      <c r="B7" s="13">
         <v>46085.0</v>
       </c>
       <c r="C7" s="4">
         <v>0.7083333333333334</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="11" t="s">
-        <v>215</v>
+      <c r="I7" s="12" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="13">
         <v>46086.0</v>
       </c>
       <c r="C8" s="8">
@@ -2982,7 +3000,7 @@
         <v>15</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>32</v>
@@ -2991,14 +3009,14 @@
         <v>65</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="B9" s="12">
+        <v>221</v>
+      </c>
+      <c r="B9" s="13">
         <v>46097.0</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -3014,7 +3032,7 @@
         <v>135</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>35</v>
@@ -3025,9 +3043,9 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="B10" s="12">
+        <v>223</v>
+      </c>
+      <c r="B10" s="13">
         <v>46111.0</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -3043,7 +3061,7 @@
         <v>142</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>185</v>
@@ -3054,9 +3072,9 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="B11" s="12">
+        <v>225</v>
+      </c>
+      <c r="B11" s="13">
         <v>46132.0</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -3069,7 +3087,7 @@
         <v>15</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>71</v>
@@ -3083,9 +3101,9 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="B12" s="12">
+        <v>227</v>
+      </c>
+      <c r="B12" s="13">
         <v>46146.0</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -3101,7 +3119,7 @@
         <v>45</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>35</v>
@@ -3114,7 +3132,7 @@
       <c r="A13" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="13">
         <v>46160.0</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -3141,9 +3159,9 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="B14" s="12">
+        <v>229</v>
+      </c>
+      <c r="B14" s="13">
         <v>46174.0</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -3156,7 +3174,7 @@
         <v>15</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>32</v>
@@ -3169,107 +3187,108 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="B15" s="14">
+      <c r="A15" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="B15" s="15">
         <v>46086.0</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="16">
         <v>0.7083333333333334</v>
       </c>
-      <c r="D15" s="16" t="s">
-        <v>229</v>
-      </c>
-      <c r="E15" s="17" t="s">
+      <c r="D15" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="E15" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="F15" s="18" t="s">
-        <v>230</v>
-      </c>
-      <c r="G15" s="17" t="s">
-        <v>231</v>
-      </c>
-      <c r="H15" s="19" t="s">
-        <v>232</v>
-      </c>
-      <c r="I15" s="20" t="s">
+      <c r="F15" s="19" t="s">
         <v>233</v>
       </c>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="13"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="13"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="13"/>
-      <c r="Q15" s="13"/>
-      <c r="R15" s="13"/>
-      <c r="S15" s="13"/>
-      <c r="T15" s="13"/>
-      <c r="U15" s="13"/>
-      <c r="V15" s="13"/>
-      <c r="W15" s="13"/>
-      <c r="X15" s="13"/>
-      <c r="Y15" s="13"/>
-      <c r="Z15" s="13"/>
+      <c r="G15" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="H15" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="I15" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="J15" s="14"/>
+      <c r="K15" s="14"/>
+      <c r="L15" s="14"/>
+      <c r="M15" s="14"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="14"/>
+      <c r="P15" s="14"/>
+      <c r="Q15" s="14"/>
+      <c r="R15" s="14"/>
+      <c r="S15" s="14"/>
+      <c r="T15" s="14"/>
+      <c r="U15" s="14"/>
+      <c r="V15" s="14"/>
+      <c r="W15" s="14"/>
+      <c r="X15" s="14"/>
+      <c r="Y15" s="14"/>
+      <c r="Z15" s="14"/>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="B16" s="15">
+        <v>46098.0</v>
+      </c>
+      <c r="C16" s="22">
+        <v>0.75</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>238</v>
+      </c>
+      <c r="G16" s="18" t="s">
         <v>234</v>
       </c>
-      <c r="B16" s="14">
-        <v>46098.0</v>
-      </c>
-      <c r="C16" s="21">
-        <v>0.75</v>
-      </c>
-      <c r="D16" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="F16" s="22" t="s">
-        <v>235</v>
-      </c>
-      <c r="G16" s="17" t="s">
-        <v>231</v>
-      </c>
-      <c r="H16" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="I16" s="24" t="s">
-        <v>236</v>
-      </c>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="13"/>
-      <c r="O16" s="13"/>
-      <c r="P16" s="13"/>
-      <c r="Q16" s="13"/>
-      <c r="R16" s="13"/>
-      <c r="S16" s="13"/>
-      <c r="T16" s="13"/>
-      <c r="U16" s="13"/>
-      <c r="V16" s="13"/>
-      <c r="W16" s="13"/>
-      <c r="X16" s="13"/>
-      <c r="Y16" s="13"/>
-      <c r="Z16" s="13"/>
+      <c r="H16" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="I16" s="25" t="s">
+        <v>239</v>
+      </c>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="14"/>
+      <c r="N16" s="14"/>
+      <c r="O16" s="14"/>
+      <c r="P16" s="14"/>
+      <c r="Q16" s="14"/>
+      <c r="R16" s="14"/>
+      <c r="S16" s="14"/>
+      <c r="T16" s="14"/>
+      <c r="U16" s="14"/>
+      <c r="V16" s="14"/>
+      <c r="W16" s="14"/>
+      <c r="X16" s="14"/>
+      <c r="Y16" s="14"/>
+      <c r="Z16" s="14"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="I2"/>
     <hyperlink r:id="rId2" ref="I3"/>
-    <hyperlink r:id="rId3" ref="I6"/>
-    <hyperlink r:id="rId4" ref="I7"/>
-    <hyperlink r:id="rId5" ref="I8"/>
-    <hyperlink r:id="rId6" ref="I15"/>
-    <hyperlink r:id="rId7" ref="I16"/>
+    <hyperlink r:id="rId3" ref="I5"/>
+    <hyperlink r:id="rId4" ref="I6"/>
+    <hyperlink r:id="rId5" ref="I7"/>
+    <hyperlink r:id="rId6" ref="I8"/>
+    <hyperlink r:id="rId7" ref="I15"/>
+    <hyperlink r:id="rId8" ref="I16"/>
   </hyperlinks>
-  <drawing r:id="rId8"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>